<commit_message>
new org_card template and validation
</commit_message>
<xml_diff>
--- a/org_templates/organization_card_blank.xlsx
+++ b/org_templates/organization_card_blank.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
   <si>
     <t xml:space="preserve">№ п/п</t>
   </si>
@@ -199,6 +199,12 @@
   </si>
   <si>
     <t xml:space="preserve">Руководитель организации (должность, Ф.И.О. полностью)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Должность</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ф.И.О.</t>
   </si>
   <si>
     <t xml:space="preserve">Председатель рабочей группы по проведению оценки профессиональных рисков (должность, Ф.И.О. полностью)</t>
@@ -245,6 +251,13 @@
       <charset val="204"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -257,13 +270,6 @@
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
       <charset val="204"/>
     </font>
     <font>
@@ -283,16 +289,14 @@
       <charset val="204"/>
     </font>
     <font>
-      <u val="single"/>
       <sz val="12"/>
-      <color rgb="FF0563C1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
       <sz val="12"/>
-      <color rgb="FF0000FF"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
@@ -376,7 +380,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -389,27 +393,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -417,19 +425,27 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -520,153 +536,202 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="42.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="61.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="76.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="40.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="4" width="40.85"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+    <row r="1" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="n">
+      <c r="D1" s="6"/>
+    </row>
+    <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="8"/>
-    </row>
-    <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="n">
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+    </row>
+    <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="8"/>
-    </row>
-    <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="n">
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+    </row>
+    <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="10"/>
-    </row>
-    <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="n">
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+    </row>
+    <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="10"/>
-    </row>
-    <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="n">
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+    </row>
+    <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="10"/>
-    </row>
-    <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="n">
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+    </row>
+    <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="10"/>
-    </row>
-    <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="n">
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+    </row>
+    <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="11"/>
-    </row>
-    <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="n">
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+    </row>
+    <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="10"/>
-    </row>
-    <row r="10" customFormat="false" ht="56.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="n">
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+    </row>
+    <row r="10" customFormat="false" ht="56.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="8"/>
-    </row>
-    <row r="11" customFormat="false" ht="56.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="n">
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+    </row>
+    <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="12"/>
-    </row>
-    <row r="12" customFormat="false" ht="56.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="n">
+      <c r="C11" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="42.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="16"/>
+    </row>
+    <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B13" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="12"/>
-    </row>
-    <row r="13" customFormat="false" ht="56.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="n">
+      <c r="D13" s="15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="42.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="16"/>
+    </row>
+    <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B15" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="13"/>
-    </row>
-    <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="14"/>
-    </row>
-    <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="15"/>
-    </row>
-    <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="14"/>
-    </row>
-    <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="19" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="32" customFormat="false" ht="8.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="33" customFormat="false" ht="14.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    </row>
+    <row r="16" customFormat="false" ht="42.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="16"/>
+    </row>
+    <row r="17" customFormat="false" ht="42.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="17"/>
+    </row>
+    <row r="18" customFormat="false" ht="42.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="18"/>
+    </row>
+    <row r="19" customFormat="false" ht="42.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="17"/>
+    </row>
   </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>